<commit_message>
update mapping Modele V3 - FHIR (#453)
* update mapping Modele V3 - FHIR

* healthcareService meta.comment n'existe pas

* test

* test

* test

* test

* Update mapping.md

* RORPractitioner.fsh test  \n

* Update RORPractitioner.fsh

* forcer le saut de ligne avec 2 espaces

* update mapping

* DivisionTerritoriale : préciser les types attendus pour les offres et les EG (#458)

* DivisionTerritoriale : préciser les types attendus pour les offres et les EG

* Update RORHealthcareService.fsh

* Update ROROrganization.fsh

* contrainte sortie de la description b62530d3c5e0b199c57f8f577237f5cab78443da
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-ror-available-time-effective-opening-closing-date.xlsx
+++ b/main/ig/StructureDefinition-ror-available-time-effective-opening-closing-date.xlsx
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-21T15:54:27+00:00</t>
+    <t>2026-01-30T10:12:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -393,7 +393,7 @@
 per-1</t>
   </si>
   <si>
-    <t>debutDateEffective</t>
+    <t>heureDebut</t>
   </si>
   <si>
     <t>./low</t>
@@ -417,7 +417,7 @@
     <t>Period.end</t>
   </si>
   <si>
-    <t>finDateEffective</t>
+    <t>heureFin</t>
   </si>
   <si>
     <t>./high</t>

</xml_diff>